<commit_message>
Add Random Forest and XGBoost Classifiers To the Study
</commit_message>
<xml_diff>
--- a/Results and Summary/CSCI 485 Final Project.xlsx
+++ b/Results and Summary/CSCI 485 Final Project.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/83d3d0baac882484/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Afolabi Soetan\Downloads\New folder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E60F0263-EC01-439C-9096-75AD8011E863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D33383B-BF29-4E58-B1C3-36F9FF737DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{AE118680-53F8-4A27-8AA4-2F3A3E8EE08C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="65">
   <si>
     <t>Iteration</t>
   </si>
@@ -159,6 +159,78 @@
   </si>
   <si>
     <t>Full Set LR vs NB</t>
+  </si>
+  <si>
+    <t>RF (PCA Only Set)</t>
+  </si>
+  <si>
+    <t>RF (Full Set)</t>
+  </si>
+  <si>
+    <t>PCA Only vs Full Data Set Comparison For RF</t>
+  </si>
+  <si>
+    <t>XGBoost (Full Set)</t>
+  </si>
+  <si>
+    <t>XGBoost (PCA Only Set)</t>
+  </si>
+  <si>
+    <t>PCA Only vs Full Data Set Comparison For XGBoost</t>
+  </si>
+  <si>
+    <t>PCA Only Set RF vs LR</t>
+  </si>
+  <si>
+    <t>Full Set RF vs LR</t>
+  </si>
+  <si>
+    <t>PCA Only Set RF vs KNN</t>
+  </si>
+  <si>
+    <t>Full Set RF vs KNN</t>
+  </si>
+  <si>
+    <t>PCA Only Set RF vs NB</t>
+  </si>
+  <si>
+    <t>Full Set RF vs NB</t>
+  </si>
+  <si>
+    <t>PCA Only Set RF vs Linear SVC</t>
+  </si>
+  <si>
+    <t>Full Set RF vs Linear SVC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCA Only Set RF vs XGBoost </t>
+  </si>
+  <si>
+    <t>Full Set RF vs XGBoost</t>
+  </si>
+  <si>
+    <t>PCA Only Set XGBoost vs LR</t>
+  </si>
+  <si>
+    <t>PCA Only Set XGBoost vs KNN</t>
+  </si>
+  <si>
+    <t>Full Set XGBoost vs LR</t>
+  </si>
+  <si>
+    <t>Full Set XGBoost vs KNN</t>
+  </si>
+  <si>
+    <t>PCA Only Set XGBoost vs NB</t>
+  </si>
+  <si>
+    <t>Full Set XGBoost vs NB</t>
+  </si>
+  <si>
+    <t>PCA Only Set XGBoost vs Linear SVC</t>
+  </si>
+  <si>
+    <t>Full Set XGBoost vs Linear SVC</t>
   </si>
 </sst>
 </file>
@@ -584,11 +656,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0AA43B4-241B-4DF1-88D9-A26C1E35E08E}">
-  <dimension ref="A1:Q266"/>
+  <dimension ref="A1:Q502"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="44.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23.42578125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="68.5703125" bestFit="1" customWidth="1"/>
@@ -2678,7 +2750,7 @@
         <v>5</v>
       </c>
       <c r="B145">
-        <v>9044</v>
+        <v>0.90439999999999998</v>
       </c>
       <c r="F145" s="2" t="s">
         <v>5</v>
@@ -3775,7 +3847,7 @@
         <v>0.82934693877550969</v>
       </c>
     </row>
-    <row r="257" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>9</v>
       </c>
@@ -3795,7 +3867,7 @@
         <v>2.2451949618693414E-3</v>
       </c>
     </row>
-    <row r="258" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>10</v>
       </c>
@@ -3815,7 +3887,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="259" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>11</v>
       </c>
@@ -3829,7 +3901,7 @@
         <v>0.68261306283880874</v>
       </c>
     </row>
-    <row r="260" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>12</v>
       </c>
@@ -3843,7 +3915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>13</v>
       </c>
@@ -3857,7 +3929,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="262" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>14</v>
       </c>
@@ -3871,7 +3943,7 @@
         <v>-23.041897217172611</v>
       </c>
     </row>
-    <row r="263" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>15</v>
       </c>
@@ -3885,7 +3957,7 @@
         <v>1.7123666326889875E-20</v>
       </c>
     </row>
-    <row r="264" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>16</v>
       </c>
@@ -3899,7 +3971,7 @@
         <v>1.6991270265334986</v>
       </c>
     </row>
-    <row r="265" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>17</v>
       </c>
@@ -3913,7 +3985,7 @@
         <v>3.4247332653779749E-20</v>
       </c>
     </row>
-    <row r="266" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A266" s="3" t="s">
         <v>18</v>
       </c>
@@ -3928,6 +4000,2959 @@
         <v>2.0452296421327048</v>
       </c>
       <c r="H266" s="3"/>
+    </row>
+    <row r="271" spans="1:15" ht="21" x14ac:dyDescent="0.35">
+      <c r="A271" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F271" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O271" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="272" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A272" t="s">
+        <v>0</v>
+      </c>
+      <c r="B272" t="s">
+        <v>22</v>
+      </c>
+      <c r="F272" t="s">
+        <v>0</v>
+      </c>
+      <c r="G272" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="273" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A273">
+        <v>1</v>
+      </c>
+      <c r="B273">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="F273">
+        <v>1</v>
+      </c>
+      <c r="G273">
+        <v>0.77551020408163196</v>
+      </c>
+    </row>
+    <row r="274" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A274">
+        <v>2</v>
+      </c>
+      <c r="B274">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="F274">
+        <v>2</v>
+      </c>
+      <c r="G274">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="O274" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="275" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A275">
+        <v>3</v>
+      </c>
+      <c r="B275">
+        <v>0.81632653061224403</v>
+      </c>
+      <c r="F275">
+        <v>3</v>
+      </c>
+      <c r="G275">
+        <v>0.79591836734693799</v>
+      </c>
+    </row>
+    <row r="276" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A276">
+        <v>4</v>
+      </c>
+      <c r="B276">
+        <v>0.79591836734693799</v>
+      </c>
+      <c r="F276">
+        <v>4</v>
+      </c>
+      <c r="G276">
+        <v>0.79591836734693799</v>
+      </c>
+      <c r="O276" s="4"/>
+      <c r="P276" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q276" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="277" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A277">
+        <v>5</v>
+      </c>
+      <c r="B277">
+        <v>0.83673469387755095</v>
+      </c>
+      <c r="F277">
+        <v>5</v>
+      </c>
+      <c r="G277">
+        <v>0.83673469387755095</v>
+      </c>
+      <c r="O277" t="s">
+        <v>5</v>
+      </c>
+      <c r="P277">
+        <v>0.7865442176870745</v>
+      </c>
+      <c r="Q277">
+        <v>0.78857142857142803</v>
+      </c>
+    </row>
+    <row r="278" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A278">
+        <v>6</v>
+      </c>
+      <c r="B278">
+        <v>0.8</v>
+      </c>
+      <c r="F278">
+        <v>6</v>
+      </c>
+      <c r="G278">
+        <v>0.82</v>
+      </c>
+      <c r="O278" t="s">
+        <v>9</v>
+      </c>
+      <c r="P278">
+        <v>2.1577386816795715E-3</v>
+      </c>
+      <c r="Q278">
+        <v>2.2409513277513739E-3</v>
+      </c>
+    </row>
+    <row r="279" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A279">
+        <v>7</v>
+      </c>
+      <c r="B279">
+        <v>0.78</v>
+      </c>
+      <c r="F279">
+        <v>7</v>
+      </c>
+      <c r="G279">
+        <v>0.78</v>
+      </c>
+      <c r="O279" t="s">
+        <v>10</v>
+      </c>
+      <c r="P279">
+        <v>30</v>
+      </c>
+      <c r="Q279">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="280" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A280">
+        <v>8</v>
+      </c>
+      <c r="B280">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="F280">
+        <v>8</v>
+      </c>
+      <c r="G280">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="O280" t="s">
+        <v>11</v>
+      </c>
+      <c r="P280">
+        <v>0.9392283929900308</v>
+      </c>
+    </row>
+    <row r="281" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A281">
+        <v>9</v>
+      </c>
+      <c r="B281">
+        <v>0.79591836734693799</v>
+      </c>
+      <c r="F281">
+        <v>9</v>
+      </c>
+      <c r="G281">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="O281" t="s">
+        <v>12</v>
+      </c>
+      <c r="P281">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="282" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A282">
+        <v>10</v>
+      </c>
+      <c r="B282">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="F282">
+        <v>10</v>
+      </c>
+      <c r="G282">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="O282" t="s">
+        <v>13</v>
+      </c>
+      <c r="P282">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="283" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A283">
+        <v>11</v>
+      </c>
+      <c r="B283">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="F283">
+        <v>11</v>
+      </c>
+      <c r="G283">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="O283" t="s">
+        <v>14</v>
+      </c>
+      <c r="P283">
+        <v>-0.67818436637832213</v>
+      </c>
+    </row>
+    <row r="284" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A284">
+        <v>12</v>
+      </c>
+      <c r="B284">
+        <v>0.79591836734693799</v>
+      </c>
+      <c r="F284">
+        <v>12</v>
+      </c>
+      <c r="G284">
+        <v>0.79591836734693799</v>
+      </c>
+      <c r="O284" t="s">
+        <v>15</v>
+      </c>
+      <c r="P284">
+        <v>0.25151537863044204</v>
+      </c>
+    </row>
+    <row r="285" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A285">
+        <v>13</v>
+      </c>
+      <c r="B285">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="F285">
+        <v>13</v>
+      </c>
+      <c r="G285">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="O285" t="s">
+        <v>16</v>
+      </c>
+      <c r="P285">
+        <v>1.6991270265334986</v>
+      </c>
+    </row>
+    <row r="286" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A286">
+        <v>14</v>
+      </c>
+      <c r="B286">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="F286">
+        <v>14</v>
+      </c>
+      <c r="G286">
+        <v>0.79591836734693799</v>
+      </c>
+      <c r="O286" t="s">
+        <v>17</v>
+      </c>
+      <c r="P286">
+        <v>0.50303075726088409</v>
+      </c>
+    </row>
+    <row r="287" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A287">
+        <v>15</v>
+      </c>
+      <c r="B287">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="F287">
+        <v>15</v>
+      </c>
+      <c r="G287">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="O287" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="P287" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="Q287" s="3"/>
+    </row>
+    <row r="288" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A288">
+        <v>16</v>
+      </c>
+      <c r="B288">
+        <v>0.84</v>
+      </c>
+      <c r="F288">
+        <v>16</v>
+      </c>
+      <c r="G288">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="289" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A289">
+        <v>17</v>
+      </c>
+      <c r="B289">
+        <v>0.78</v>
+      </c>
+      <c r="F289">
+        <v>17</v>
+      </c>
+      <c r="G289">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="290" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A290">
+        <v>18</v>
+      </c>
+      <c r="B290">
+        <v>0.85714285714285698</v>
+      </c>
+      <c r="F290">
+        <v>18</v>
+      </c>
+      <c r="G290">
+        <v>0.87755102040816302</v>
+      </c>
+    </row>
+    <row r="291" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A291">
+        <v>19</v>
+      </c>
+      <c r="B291">
+        <v>0.71428571428571397</v>
+      </c>
+      <c r="F291">
+        <v>19</v>
+      </c>
+      <c r="G291">
+        <v>0.71428571428571397</v>
+      </c>
+    </row>
+    <row r="292" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A292">
+        <v>20</v>
+      </c>
+      <c r="B292">
+        <v>0.79591836734693799</v>
+      </c>
+      <c r="F292">
+        <v>20</v>
+      </c>
+      <c r="G292">
+        <v>0.79591836734693799</v>
+      </c>
+    </row>
+    <row r="293" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A293">
+        <v>21</v>
+      </c>
+      <c r="B293">
+        <v>0.83673469387755095</v>
+      </c>
+      <c r="F293">
+        <v>21</v>
+      </c>
+      <c r="G293">
+        <v>0.83673469387755095</v>
+      </c>
+    </row>
+    <row r="294" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A294">
+        <v>22</v>
+      </c>
+      <c r="B294">
+        <v>0.73469387755102</v>
+      </c>
+      <c r="F294">
+        <v>22</v>
+      </c>
+      <c r="G294">
+        <v>0.71428571428571397</v>
+      </c>
+    </row>
+    <row r="295" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A295">
+        <v>23</v>
+      </c>
+      <c r="B295">
+        <v>0.73469387755102</v>
+      </c>
+      <c r="F295">
+        <v>23</v>
+      </c>
+      <c r="G295">
+        <v>0.73469387755102</v>
+      </c>
+    </row>
+    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A296">
+        <v>24</v>
+      </c>
+      <c r="B296">
+        <v>0.91836734693877498</v>
+      </c>
+      <c r="F296">
+        <v>24</v>
+      </c>
+      <c r="G296">
+        <v>0.89795918367346905</v>
+      </c>
+    </row>
+    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A297">
+        <v>25</v>
+      </c>
+      <c r="B297">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="F297">
+        <v>25</v>
+      </c>
+      <c r="G297">
+        <v>0.75510204081632604</v>
+      </c>
+    </row>
+    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A298">
+        <v>26</v>
+      </c>
+      <c r="B298">
+        <v>0.8</v>
+      </c>
+      <c r="F298">
+        <v>26</v>
+      </c>
+      <c r="G298">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A299">
+        <v>27</v>
+      </c>
+      <c r="B299">
+        <v>0.78</v>
+      </c>
+      <c r="F299">
+        <v>27</v>
+      </c>
+      <c r="G299">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="300" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A300">
+        <v>28</v>
+      </c>
+      <c r="B300">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="F300">
+        <v>28</v>
+      </c>
+      <c r="G300">
+        <v>0.75510204081632604</v>
+      </c>
+    </row>
+    <row r="301" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A301">
+        <v>29</v>
+      </c>
+      <c r="B301">
+        <v>0.69387755102040805</v>
+      </c>
+      <c r="F301">
+        <v>29</v>
+      </c>
+      <c r="G301">
+        <v>0.73469387755102</v>
+      </c>
+    </row>
+    <row r="302" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A302">
+        <v>30</v>
+      </c>
+      <c r="B302">
+        <v>0.85714285714285698</v>
+      </c>
+      <c r="F302">
+        <v>30</v>
+      </c>
+      <c r="G302">
+        <v>0.89795918367346905</v>
+      </c>
+    </row>
+    <row r="303" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A303" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B303">
+        <v>0.78859999999999997</v>
+      </c>
+      <c r="F303" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G303">
+        <v>0.78649999999999998</v>
+      </c>
+    </row>
+    <row r="306" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+      <c r="A306" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F306" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="O306" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="308" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A308" t="s">
+        <v>0</v>
+      </c>
+      <c r="B308" t="s">
+        <v>1</v>
+      </c>
+      <c r="F308" t="s">
+        <v>0</v>
+      </c>
+      <c r="G308" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="309" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A309">
+        <v>1</v>
+      </c>
+      <c r="B309">
+        <v>0.79591836734693799</v>
+      </c>
+      <c r="F309">
+        <v>1</v>
+      </c>
+      <c r="G309">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="O309" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="310" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A310">
+        <v>2</v>
+      </c>
+      <c r="B310">
+        <v>0.83673469387755095</v>
+      </c>
+      <c r="F310">
+        <v>2</v>
+      </c>
+      <c r="G310">
+        <v>0.79591836734693799</v>
+      </c>
+    </row>
+    <row r="311" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A311">
+        <v>3</v>
+      </c>
+      <c r="B311">
+        <v>0.85714285714285698</v>
+      </c>
+      <c r="F311">
+        <v>3</v>
+      </c>
+      <c r="G311">
+        <v>0.87755102040816302</v>
+      </c>
+      <c r="O311" s="4"/>
+      <c r="P311" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q311" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="312" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A312">
+        <v>4</v>
+      </c>
+      <c r="B312">
+        <v>0.81632653061224403</v>
+      </c>
+      <c r="F312">
+        <v>4</v>
+      </c>
+      <c r="G312">
+        <v>0.83673469387755095</v>
+      </c>
+      <c r="O312" t="s">
+        <v>5</v>
+      </c>
+      <c r="P312">
+        <v>0.82247619047619003</v>
+      </c>
+      <c r="Q312">
+        <v>0.81838095238095199</v>
+      </c>
+    </row>
+    <row r="313" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A313">
+        <v>5</v>
+      </c>
+      <c r="B313">
+        <v>0.83673469387755095</v>
+      </c>
+      <c r="F313">
+        <v>5</v>
+      </c>
+      <c r="G313">
+        <v>0.83673469387755095</v>
+      </c>
+      <c r="O313" t="s">
+        <v>9</v>
+      </c>
+      <c r="P313">
+        <v>2.4659372770924073E-3</v>
+      </c>
+      <c r="Q313">
+        <v>2.7039823445212121E-3</v>
+      </c>
+    </row>
+    <row r="314" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A314">
+        <v>6</v>
+      </c>
+      <c r="B314">
+        <v>0.86</v>
+      </c>
+      <c r="F314">
+        <v>6</v>
+      </c>
+      <c r="G314">
+        <v>0.86</v>
+      </c>
+      <c r="O314" t="s">
+        <v>10</v>
+      </c>
+      <c r="P314">
+        <v>30</v>
+      </c>
+      <c r="Q314">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="315" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A315">
+        <v>7</v>
+      </c>
+      <c r="B315">
+        <v>0.8</v>
+      </c>
+      <c r="F315">
+        <v>7</v>
+      </c>
+      <c r="G315">
+        <v>0.8</v>
+      </c>
+      <c r="O315" t="s">
+        <v>11</v>
+      </c>
+      <c r="P315">
+        <v>0.93800963719948172</v>
+      </c>
+    </row>
+    <row r="316" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A316">
+        <v>8</v>
+      </c>
+      <c r="B316">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="F316">
+        <v>8</v>
+      </c>
+      <c r="G316">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="O316" t="s">
+        <v>12</v>
+      </c>
+      <c r="P316">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="317" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A317">
+        <v>9</v>
+      </c>
+      <c r="B317">
+        <v>0.83673469387755095</v>
+      </c>
+      <c r="F317">
+        <v>9</v>
+      </c>
+      <c r="G317">
+        <v>0.85714285714285698</v>
+      </c>
+      <c r="O317" t="s">
+        <v>13</v>
+      </c>
+      <c r="P317">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="318" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A318">
+        <v>10</v>
+      </c>
+      <c r="B318">
+        <v>0.79591836734693799</v>
+      </c>
+      <c r="F318">
+        <v>10</v>
+      </c>
+      <c r="G318">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="O318" t="s">
+        <v>14</v>
+      </c>
+      <c r="P318">
+        <v>1.2430213298792068</v>
+      </c>
+    </row>
+    <row r="319" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A319">
+        <v>11</v>
+      </c>
+      <c r="B319">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="F319">
+        <v>11</v>
+      </c>
+      <c r="G319">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="O319" t="s">
+        <v>15</v>
+      </c>
+      <c r="P319">
+        <v>0.11190819598656337</v>
+      </c>
+    </row>
+    <row r="320" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A320">
+        <v>12</v>
+      </c>
+      <c r="B320">
+        <v>0.81632653061224403</v>
+      </c>
+      <c r="F320">
+        <v>12</v>
+      </c>
+      <c r="G320">
+        <v>0.83673469387755095</v>
+      </c>
+      <c r="O320" t="s">
+        <v>16</v>
+      </c>
+      <c r="P320">
+        <v>1.6991270265334986</v>
+      </c>
+    </row>
+    <row r="321" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A321">
+        <v>13</v>
+      </c>
+      <c r="B321">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="F321">
+        <v>13</v>
+      </c>
+      <c r="G321">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="O321" t="s">
+        <v>17</v>
+      </c>
+      <c r="P321">
+        <v>0.22381639197312675</v>
+      </c>
+    </row>
+    <row r="322" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A322">
+        <v>14</v>
+      </c>
+      <c r="B322">
+        <v>0.93877551020408101</v>
+      </c>
+      <c r="F322">
+        <v>14</v>
+      </c>
+      <c r="G322">
+        <v>0.89795918367346905</v>
+      </c>
+      <c r="O322" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="P322" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="Q322" s="3"/>
+    </row>
+    <row r="323" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A323">
+        <v>15</v>
+      </c>
+      <c r="B323">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="F323">
+        <v>15</v>
+      </c>
+      <c r="G323">
+        <v>0.77551020408163196</v>
+      </c>
+    </row>
+    <row r="324" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A324">
+        <v>16</v>
+      </c>
+      <c r="B324">
+        <v>0.86</v>
+      </c>
+      <c r="F324">
+        <v>16</v>
+      </c>
+      <c r="G324">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="325" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A325">
+        <v>17</v>
+      </c>
+      <c r="B325">
+        <v>0.8</v>
+      </c>
+      <c r="F325">
+        <v>17</v>
+      </c>
+      <c r="G325">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="326" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A326">
+        <v>18</v>
+      </c>
+      <c r="B326">
+        <v>0.89795918367346905</v>
+      </c>
+      <c r="F326">
+        <v>18</v>
+      </c>
+      <c r="G326">
+        <v>0.91836734693877498</v>
+      </c>
+    </row>
+    <row r="327" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A327">
+        <v>19</v>
+      </c>
+      <c r="B327">
+        <v>0.77551020408163196</v>
+      </c>
+      <c r="F327">
+        <v>19</v>
+      </c>
+      <c r="G327">
+        <v>0.77551020408163196</v>
+      </c>
+    </row>
+    <row r="328" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A328">
+        <v>20</v>
+      </c>
+      <c r="B328">
+        <v>0.81632653061224403</v>
+      </c>
+      <c r="F328">
+        <v>20</v>
+      </c>
+      <c r="G328">
+        <v>0.81632653061224403</v>
+      </c>
+    </row>
+    <row r="329" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A329">
+        <v>21</v>
+      </c>
+      <c r="B329">
+        <v>0.85714285714285698</v>
+      </c>
+      <c r="F329">
+        <v>21</v>
+      </c>
+      <c r="G329">
+        <v>0.85714285714285698</v>
+      </c>
+    </row>
+    <row r="330" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A330">
+        <v>22</v>
+      </c>
+      <c r="B330">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="F330">
+        <v>22</v>
+      </c>
+      <c r="G330">
+        <v>0.73469387755102</v>
+      </c>
+    </row>
+    <row r="331" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A331">
+        <v>23</v>
+      </c>
+      <c r="B331">
+        <v>0.81632653061224403</v>
+      </c>
+      <c r="F331">
+        <v>23</v>
+      </c>
+      <c r="G331">
+        <v>0.81632653061224403</v>
+      </c>
+    </row>
+    <row r="332" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A332">
+        <v>24</v>
+      </c>
+      <c r="B332">
+        <v>0.93877551020408101</v>
+      </c>
+      <c r="F332">
+        <v>24</v>
+      </c>
+      <c r="G332">
+        <v>0.91836734693877498</v>
+      </c>
+    </row>
+    <row r="333" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A333">
+        <v>25</v>
+      </c>
+      <c r="B333">
+        <v>0.79591836734693799</v>
+      </c>
+      <c r="F333">
+        <v>25</v>
+      </c>
+      <c r="G333">
+        <v>0.79591836734693799</v>
+      </c>
+    </row>
+    <row r="334" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A334">
+        <v>26</v>
+      </c>
+      <c r="B334">
+        <v>0.8</v>
+      </c>
+      <c r="F334">
+        <v>26</v>
+      </c>
+      <c r="G334">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="335" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A335">
+        <v>27</v>
+      </c>
+      <c r="B335">
+        <v>0.84</v>
+      </c>
+      <c r="F335">
+        <v>27</v>
+      </c>
+      <c r="G335">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="336" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A336">
+        <v>28</v>
+      </c>
+      <c r="B336">
+        <v>0.79591836734693799</v>
+      </c>
+      <c r="F336">
+        <v>28</v>
+      </c>
+      <c r="G336">
+        <v>0.77551020408163196</v>
+      </c>
+    </row>
+    <row r="337" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A337">
+        <v>29</v>
+      </c>
+      <c r="B337">
+        <v>0.75510204081632604</v>
+      </c>
+      <c r="F337">
+        <v>29</v>
+      </c>
+      <c r="G337">
+        <v>0.73469387755102</v>
+      </c>
+    </row>
+    <row r="338" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A338">
+        <v>30</v>
+      </c>
+      <c r="B338">
+        <v>0.89795918367346905</v>
+      </c>
+      <c r="F338">
+        <v>30</v>
+      </c>
+      <c r="G338">
+        <v>0.87755102040816302</v>
+      </c>
+    </row>
+    <row r="339" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A339" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B339">
+        <v>0.81840000000000002</v>
+      </c>
+      <c r="F339" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G339">
+        <v>0.82250000000000001</v>
+      </c>
+    </row>
+    <row r="343" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+      <c r="A343" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F343" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="345" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A345" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F345" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="346" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="347" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A347" s="4"/>
+      <c r="B347" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C347" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F347" s="4"/>
+      <c r="G347" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H347" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="348" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A348" t="s">
+        <v>5</v>
+      </c>
+      <c r="B348">
+        <v>0.78857142857142803</v>
+      </c>
+      <c r="C348">
+        <v>0.6144489795918362</v>
+      </c>
+      <c r="F348" t="s">
+        <v>5</v>
+      </c>
+      <c r="G348">
+        <v>0.7865442176870745</v>
+      </c>
+      <c r="H348">
+        <v>0.61987755102040754</v>
+      </c>
+    </row>
+    <row r="349" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A349" t="s">
+        <v>9</v>
+      </c>
+      <c r="B349">
+        <v>2.2409513277513739E-3</v>
+      </c>
+      <c r="C349">
+        <v>5.1733340992979309E-3</v>
+      </c>
+      <c r="F349" t="s">
+        <v>9</v>
+      </c>
+      <c r="G349">
+        <v>2.1577386816795715E-3</v>
+      </c>
+      <c r="H349">
+        <v>4.6410564563617949E-3</v>
+      </c>
+    </row>
+    <row r="350" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A350" t="s">
+        <v>10</v>
+      </c>
+      <c r="B350">
+        <v>30</v>
+      </c>
+      <c r="C350">
+        <v>30</v>
+      </c>
+      <c r="F350" t="s">
+        <v>10</v>
+      </c>
+      <c r="G350">
+        <v>30</v>
+      </c>
+      <c r="H350">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="351" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A351" t="s">
+        <v>11</v>
+      </c>
+      <c r="B351">
+        <v>0.66767672284608615</v>
+      </c>
+      <c r="F351" t="s">
+        <v>11</v>
+      </c>
+      <c r="G351">
+        <v>0.72153042254735422</v>
+      </c>
+    </row>
+    <row r="352" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A352" t="s">
+        <v>12</v>
+      </c>
+      <c r="B352">
+        <v>0</v>
+      </c>
+      <c r="F352" t="s">
+        <v>12</v>
+      </c>
+      <c r="G352">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="353" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A353" t="s">
+        <v>13</v>
+      </c>
+      <c r="B353">
+        <v>29</v>
+      </c>
+      <c r="F353" t="s">
+        <v>13</v>
+      </c>
+      <c r="G353">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="354" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A354" t="s">
+        <v>14</v>
+      </c>
+      <c r="B354">
+        <v>17.809770671466158</v>
+      </c>
+      <c r="F354" t="s">
+        <v>14</v>
+      </c>
+      <c r="G354">
+        <v>19.321587547085407</v>
+      </c>
+    </row>
+    <row r="355" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A355" t="s">
+        <v>15</v>
+      </c>
+      <c r="B355">
+        <v>1.8554163619824876E-17</v>
+      </c>
+      <c r="F355" t="s">
+        <v>15</v>
+      </c>
+      <c r="G355">
+        <v>2.0871550953827062E-18</v>
+      </c>
+    </row>
+    <row r="356" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A356" t="s">
+        <v>16</v>
+      </c>
+      <c r="B356">
+        <v>1.6991270265334986</v>
+      </c>
+      <c r="F356" t="s">
+        <v>16</v>
+      </c>
+      <c r="G356">
+        <v>1.6991270265334986</v>
+      </c>
+    </row>
+    <row r="357" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A357" t="s">
+        <v>17</v>
+      </c>
+      <c r="B357">
+        <v>3.7108327239649751E-17</v>
+      </c>
+      <c r="F357" t="s">
+        <v>17</v>
+      </c>
+      <c r="G357">
+        <v>4.1743101907654124E-18</v>
+      </c>
+    </row>
+    <row r="358" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A358" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B358" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="C358" s="3"/>
+      <c r="F358" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G358" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="H358" s="3"/>
+    </row>
+    <row r="361" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+      <c r="A361" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F361" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="363" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A363" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F363" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="364" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="365" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A365" s="4"/>
+      <c r="B365" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C365" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F365" s="4"/>
+      <c r="G365" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H365" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="366" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A366" t="s">
+        <v>5</v>
+      </c>
+      <c r="B366">
+        <v>0.78857142857142803</v>
+      </c>
+      <c r="C366">
+        <v>0.7749659863945576</v>
+      </c>
+      <c r="F366" t="s">
+        <v>5</v>
+      </c>
+      <c r="G366">
+        <v>0.7865442176870745</v>
+      </c>
+      <c r="H366">
+        <v>0.77293877551020373</v>
+      </c>
+    </row>
+    <row r="367" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A367" t="s">
+        <v>9</v>
+      </c>
+      <c r="B367">
+        <v>2.2409513277513739E-3</v>
+      </c>
+      <c r="C367">
+        <v>2.8502530076069833E-3</v>
+      </c>
+      <c r="F367" t="s">
+        <v>9</v>
+      </c>
+      <c r="G367">
+        <v>2.1577386816795715E-3</v>
+      </c>
+      <c r="H367">
+        <v>3.1408309755992427E-3</v>
+      </c>
+    </row>
+    <row r="368" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A368" t="s">
+        <v>10</v>
+      </c>
+      <c r="B368">
+        <v>30</v>
+      </c>
+      <c r="C368">
+        <v>30</v>
+      </c>
+      <c r="F368" t="s">
+        <v>10</v>
+      </c>
+      <c r="G368">
+        <v>30</v>
+      </c>
+      <c r="H368">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="369" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A369" t="s">
+        <v>11</v>
+      </c>
+      <c r="B369">
+        <v>0.88690917074192033</v>
+      </c>
+      <c r="F369" t="s">
+        <v>11</v>
+      </c>
+      <c r="G369">
+        <v>0.85120052360799092</v>
+      </c>
+    </row>
+    <row r="370" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A370" t="s">
+        <v>12</v>
+      </c>
+      <c r="B370">
+        <v>0</v>
+      </c>
+      <c r="F370" t="s">
+        <v>12</v>
+      </c>
+      <c r="G370">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="371" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A371" t="s">
+        <v>13</v>
+      </c>
+      <c r="B371">
+        <v>29</v>
+      </c>
+      <c r="F371" t="s">
+        <v>13</v>
+      </c>
+      <c r="G371">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="372" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A372" t="s">
+        <v>14</v>
+      </c>
+      <c r="B372">
+        <v>3.0216373742108034</v>
+      </c>
+      <c r="F372" t="s">
+        <v>14</v>
+      </c>
+      <c r="G372">
+        <v>2.5312218444049783</v>
+      </c>
+    </row>
+    <row r="373" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A373" t="s">
+        <v>15</v>
+      </c>
+      <c r="B373">
+        <v>2.6048878760313648E-3</v>
+      </c>
+      <c r="F373" t="s">
+        <v>15</v>
+      </c>
+      <c r="G373">
+        <v>8.5231943178696017E-3</v>
+      </c>
+    </row>
+    <row r="374" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A374" t="s">
+        <v>16</v>
+      </c>
+      <c r="B374">
+        <v>1.6991270265334986</v>
+      </c>
+      <c r="F374" t="s">
+        <v>16</v>
+      </c>
+      <c r="G374">
+        <v>1.6991270265334986</v>
+      </c>
+    </row>
+    <row r="375" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A375" t="s">
+        <v>17</v>
+      </c>
+      <c r="B375">
+        <v>5.2097757520627296E-3</v>
+      </c>
+      <c r="F375" t="s">
+        <v>17</v>
+      </c>
+      <c r="G375">
+        <v>1.7046388635739203E-2</v>
+      </c>
+    </row>
+    <row r="376" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A376" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B376" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="C376" s="3"/>
+      <c r="F376" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G376" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="H376" s="3"/>
+    </row>
+    <row r="379" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+      <c r="A379" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F379" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="381" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A381" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F381" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="382" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="383" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A383" s="4"/>
+      <c r="B383" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C383" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F383" s="4"/>
+      <c r="G383" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H383" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="384" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A384" t="s">
+        <v>5</v>
+      </c>
+      <c r="B384">
+        <v>0.78857142857142803</v>
+      </c>
+      <c r="C384">
+        <v>0.82934693877550969</v>
+      </c>
+      <c r="F384" t="s">
+        <v>5</v>
+      </c>
+      <c r="G384">
+        <v>0.7865442176870745</v>
+      </c>
+      <c r="H384">
+        <v>0.82934693877550969</v>
+      </c>
+    </row>
+    <row r="385" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A385" t="s">
+        <v>9</v>
+      </c>
+      <c r="B385">
+        <v>2.2409513277513739E-3</v>
+      </c>
+      <c r="C385">
+        <v>2.2451949618693414E-3</v>
+      </c>
+      <c r="F385" t="s">
+        <v>9</v>
+      </c>
+      <c r="G385">
+        <v>2.1577386816795715E-3</v>
+      </c>
+      <c r="H385">
+        <v>2.2451949618693414E-3</v>
+      </c>
+    </row>
+    <row r="386" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A386" t="s">
+        <v>10</v>
+      </c>
+      <c r="B386">
+        <v>30</v>
+      </c>
+      <c r="C386">
+        <v>30</v>
+      </c>
+      <c r="F386" t="s">
+        <v>10</v>
+      </c>
+      <c r="G386">
+        <v>30</v>
+      </c>
+      <c r="H386">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="387" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A387" t="s">
+        <v>11</v>
+      </c>
+      <c r="B387">
+        <v>0.79649964110552818</v>
+      </c>
+      <c r="F387" t="s">
+        <v>11</v>
+      </c>
+      <c r="G387">
+        <v>0.73840024560918605</v>
+      </c>
+    </row>
+    <row r="388" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A388" t="s">
+        <v>12</v>
+      </c>
+      <c r="B388">
+        <v>0</v>
+      </c>
+      <c r="F388" t="s">
+        <v>12</v>
+      </c>
+      <c r="G388">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="389" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A389" t="s">
+        <v>13</v>
+      </c>
+      <c r="B389">
+        <v>29</v>
+      </c>
+      <c r="F389" t="s">
+        <v>13</v>
+      </c>
+      <c r="G389">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="390" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A390" t="s">
+        <v>14</v>
+      </c>
+      <c r="B390">
+        <v>-7.3916321452782894</v>
+      </c>
+      <c r="F390" t="s">
+        <v>14</v>
+      </c>
+      <c r="G390">
+        <v>-6.9059173787353112</v>
+      </c>
+    </row>
+    <row r="391" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A391" t="s">
+        <v>15</v>
+      </c>
+      <c r="B391">
+        <v>1.9112428248731619E-8</v>
+      </c>
+      <c r="F391" t="s">
+        <v>15</v>
+      </c>
+      <c r="G391">
+        <v>6.8687852726130566E-8</v>
+      </c>
+    </row>
+    <row r="392" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A392" t="s">
+        <v>16</v>
+      </c>
+      <c r="B392">
+        <v>1.6991270265334986</v>
+      </c>
+      <c r="F392" t="s">
+        <v>16</v>
+      </c>
+      <c r="G392">
+        <v>1.6991270265334986</v>
+      </c>
+    </row>
+    <row r="393" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A393" t="s">
+        <v>17</v>
+      </c>
+      <c r="B393">
+        <v>3.8224856497463238E-8</v>
+      </c>
+      <c r="F393" t="s">
+        <v>17</v>
+      </c>
+      <c r="G393">
+        <v>1.3737570545226113E-7</v>
+      </c>
+    </row>
+    <row r="394" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A394" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B394" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="C394" s="3"/>
+      <c r="F394" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G394" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="H394" s="3"/>
+    </row>
+    <row r="397" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+      <c r="A397" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F397" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="399" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A399" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F399" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="400" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="401" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A401" s="4"/>
+      <c r="B401" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C401" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F401" s="4"/>
+      <c r="G401" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H401" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="402" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A402" t="s">
+        <v>5</v>
+      </c>
+      <c r="B402">
+        <v>0.78857142857142803</v>
+      </c>
+      <c r="C402">
+        <v>0.90304761904761865</v>
+      </c>
+      <c r="F402" t="s">
+        <v>5</v>
+      </c>
+      <c r="G402">
+        <v>0.7865442176870745</v>
+      </c>
+      <c r="H402">
+        <v>0.90440816326530571</v>
+      </c>
+    </row>
+    <row r="403" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A403" t="s">
+        <v>9</v>
+      </c>
+      <c r="B403">
+        <v>2.2409513277513739E-3</v>
+      </c>
+      <c r="C403">
+        <v>1.5703426254386223E-3</v>
+      </c>
+      <c r="F403" t="s">
+        <v>9</v>
+      </c>
+      <c r="G403">
+        <v>2.1577386816795715E-3</v>
+      </c>
+      <c r="H403">
+        <v>1.5541041807292822E-3</v>
+      </c>
+    </row>
+    <row r="404" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A404" t="s">
+        <v>10</v>
+      </c>
+      <c r="B404">
+        <v>30</v>
+      </c>
+      <c r="C404">
+        <v>30</v>
+      </c>
+      <c r="F404" t="s">
+        <v>10</v>
+      </c>
+      <c r="G404">
+        <v>30</v>
+      </c>
+      <c r="H404">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="405" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A405" t="s">
+        <v>11</v>
+      </c>
+      <c r="B405">
+        <v>0.64884696343467652</v>
+      </c>
+      <c r="F405" t="s">
+        <v>11</v>
+      </c>
+      <c r="G405">
+        <v>0.53702126833526653</v>
+      </c>
+    </row>
+    <row r="406" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A406" t="s">
+        <v>12</v>
+      </c>
+      <c r="B406">
+        <v>0</v>
+      </c>
+      <c r="F406" t="s">
+        <v>12</v>
+      </c>
+      <c r="G406">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="407" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A407" t="s">
+        <v>13</v>
+      </c>
+      <c r="B407">
+        <v>29</v>
+      </c>
+      <c r="F407" t="s">
+        <v>13</v>
+      </c>
+      <c r="G407">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="408" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A408" t="s">
+        <v>14</v>
+      </c>
+      <c r="B408">
+        <v>-16.89740558886982</v>
+      </c>
+      <c r="F408" t="s">
+        <v>14</v>
+      </c>
+      <c r="G408">
+        <v>-15.453931654265617</v>
+      </c>
+    </row>
+    <row r="409" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A409" t="s">
+        <v>15</v>
+      </c>
+      <c r="B409">
+        <v>7.4883488123895406E-17</v>
+      </c>
+      <c r="F409" t="s">
+        <v>15</v>
+      </c>
+      <c r="G409">
+        <v>7.7646332030637917E-16</v>
+      </c>
+    </row>
+    <row r="410" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A410" t="s">
+        <v>16</v>
+      </c>
+      <c r="B410">
+        <v>1.6991270265334986</v>
+      </c>
+      <c r="F410" t="s">
+        <v>16</v>
+      </c>
+      <c r="G410">
+        <v>1.6991270265334986</v>
+      </c>
+    </row>
+    <row r="411" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A411" t="s">
+        <v>17</v>
+      </c>
+      <c r="B411">
+        <v>1.4976697624779081E-16</v>
+      </c>
+      <c r="F411" t="s">
+        <v>17</v>
+      </c>
+      <c r="G411">
+        <v>1.5529266406127583E-15</v>
+      </c>
+    </row>
+    <row r="412" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A412" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B412" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="C412" s="3"/>
+      <c r="F412" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G412" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="H412" s="3"/>
+    </row>
+    <row r="415" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+      <c r="A415" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F415" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="417" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A417" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F417" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="418" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="419" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A419" s="4"/>
+      <c r="B419" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C419" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F419" s="4"/>
+      <c r="G419" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H419" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="420" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A420" t="s">
+        <v>5</v>
+      </c>
+      <c r="B420">
+        <v>0.78857142857142803</v>
+      </c>
+      <c r="C420">
+        <v>0.81838095238095199</v>
+      </c>
+      <c r="F420" t="s">
+        <v>5</v>
+      </c>
+      <c r="G420">
+        <v>0.7865442176870745</v>
+      </c>
+      <c r="H420">
+        <v>0.82247619047619003</v>
+      </c>
+    </row>
+    <row r="421" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A421" t="s">
+        <v>9</v>
+      </c>
+      <c r="B421">
+        <v>2.2409513277513739E-3</v>
+      </c>
+      <c r="C421">
+        <v>2.7039823445212121E-3</v>
+      </c>
+      <c r="F421" t="s">
+        <v>9</v>
+      </c>
+      <c r="G421">
+        <v>2.1577386816795715E-3</v>
+      </c>
+      <c r="H421">
+        <v>2.4659372770924073E-3</v>
+      </c>
+    </row>
+    <row r="422" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A422" t="s">
+        <v>10</v>
+      </c>
+      <c r="B422">
+        <v>30</v>
+      </c>
+      <c r="C422">
+        <v>30</v>
+      </c>
+      <c r="F422" t="s">
+        <v>10</v>
+      </c>
+      <c r="G422">
+        <v>30</v>
+      </c>
+      <c r="H422">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="423" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A423" t="s">
+        <v>11</v>
+      </c>
+      <c r="B423">
+        <v>0.79751454927920462</v>
+      </c>
+      <c r="F423" t="s">
+        <v>11</v>
+      </c>
+      <c r="G423">
+        <v>0.71841009014923818</v>
+      </c>
+    </row>
+    <row r="424" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A424" t="s">
+        <v>12</v>
+      </c>
+      <c r="B424">
+        <v>0</v>
+      </c>
+      <c r="F424" t="s">
+        <v>12</v>
+      </c>
+      <c r="G424">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="425" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A425" t="s">
+        <v>13</v>
+      </c>
+      <c r="B425">
+        <v>29</v>
+      </c>
+      <c r="F425" t="s">
+        <v>13</v>
+      </c>
+      <c r="G425">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="426" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A426" t="s">
+        <v>14</v>
+      </c>
+      <c r="B426">
+        <v>-5.1157928476354568</v>
+      </c>
+      <c r="F426" t="s">
+        <v>14</v>
+      </c>
+      <c r="G426">
+        <v>-5.4388968553218326</v>
+      </c>
+    </row>
+    <row r="427" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A427" t="s">
+        <v>15</v>
+      </c>
+      <c r="B427">
+        <v>9.1925249297954942E-6</v>
+      </c>
+      <c r="F427" t="s">
+        <v>15</v>
+      </c>
+      <c r="G427">
+        <v>3.7473777193880924E-6</v>
+      </c>
+    </row>
+    <row r="428" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A428" t="s">
+        <v>16</v>
+      </c>
+      <c r="B428">
+        <v>1.6991270265334986</v>
+      </c>
+      <c r="F428" t="s">
+        <v>16</v>
+      </c>
+      <c r="G428">
+        <v>1.6991270265334986</v>
+      </c>
+    </row>
+    <row r="429" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A429" t="s">
+        <v>17</v>
+      </c>
+      <c r="B429">
+        <v>1.8385049859590988E-5</v>
+      </c>
+      <c r="F429" t="s">
+        <v>17</v>
+      </c>
+      <c r="G429">
+        <v>7.4947554387761847E-6</v>
+      </c>
+    </row>
+    <row r="430" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A430" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B430" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="C430" s="3"/>
+      <c r="F430" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G430" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="H430" s="3"/>
+    </row>
+    <row r="433" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+      <c r="A433" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F433" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="435" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A435" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F435" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="436" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="437" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A437" s="4"/>
+      <c r="B437" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C437" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F437" s="4"/>
+      <c r="G437" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H437" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="438" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A438" t="s">
+        <v>5</v>
+      </c>
+      <c r="B438">
+        <v>0.81838095238095199</v>
+      </c>
+      <c r="C438">
+        <v>0.6144489795918362</v>
+      </c>
+      <c r="F438" t="s">
+        <v>5</v>
+      </c>
+      <c r="G438">
+        <v>0.82247619047619003</v>
+      </c>
+      <c r="H438">
+        <v>0.61987755102040754</v>
+      </c>
+    </row>
+    <row r="439" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A439" t="s">
+        <v>9</v>
+      </c>
+      <c r="B439">
+        <v>2.7039823445212121E-3</v>
+      </c>
+      <c r="C439">
+        <v>5.1733340992979309E-3</v>
+      </c>
+      <c r="F439" t="s">
+        <v>9</v>
+      </c>
+      <c r="G439">
+        <v>2.4659372770924073E-3</v>
+      </c>
+      <c r="H439">
+        <v>4.6410564563617949E-3</v>
+      </c>
+    </row>
+    <row r="440" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A440" t="s">
+        <v>10</v>
+      </c>
+      <c r="B440">
+        <v>30</v>
+      </c>
+      <c r="C440">
+        <v>30</v>
+      </c>
+      <c r="F440" t="s">
+        <v>10</v>
+      </c>
+      <c r="G440">
+        <v>30</v>
+      </c>
+      <c r="H440">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="441" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A441" t="s">
+        <v>11</v>
+      </c>
+      <c r="B441">
+        <v>0.55431702132512184</v>
+      </c>
+      <c r="F441" t="s">
+        <v>11</v>
+      </c>
+      <c r="G441">
+        <v>0.50189969789340894</v>
+      </c>
+    </row>
+    <row r="442" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A442" t="s">
+        <v>12</v>
+      </c>
+      <c r="B442">
+        <v>0</v>
+      </c>
+      <c r="F442" t="s">
+        <v>12</v>
+      </c>
+      <c r="G442">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="443" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A443" t="s">
+        <v>13</v>
+      </c>
+      <c r="B443">
+        <v>29</v>
+      </c>
+      <c r="F443" t="s">
+        <v>13</v>
+      </c>
+      <c r="G443">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="444" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A444" t="s">
+        <v>14</v>
+      </c>
+      <c r="B444">
+        <v>18.286918201518727</v>
+      </c>
+      <c r="F444" t="s">
+        <v>14</v>
+      </c>
+      <c r="G444">
+        <v>18.215550043916899</v>
+      </c>
+    </row>
+    <row r="445" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A445" t="s">
+        <v>15</v>
+      </c>
+      <c r="B445">
+        <v>9.1582385142598811E-18</v>
+      </c>
+      <c r="F445" t="s">
+        <v>15</v>
+      </c>
+      <c r="G445">
+        <v>1.0168176774318586E-17</v>
+      </c>
+    </row>
+    <row r="446" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A446" t="s">
+        <v>16</v>
+      </c>
+      <c r="B446">
+        <v>1.6991270265334986</v>
+      </c>
+      <c r="F446" t="s">
+        <v>16</v>
+      </c>
+      <c r="G446">
+        <v>1.6991270265334986</v>
+      </c>
+    </row>
+    <row r="447" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A447" t="s">
+        <v>17</v>
+      </c>
+      <c r="B447">
+        <v>1.8316477028519762E-17</v>
+      </c>
+      <c r="F447" t="s">
+        <v>17</v>
+      </c>
+      <c r="G447">
+        <v>2.0336353548637172E-17</v>
+      </c>
+    </row>
+    <row r="448" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A448" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B448" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="C448" s="3"/>
+      <c r="F448" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G448" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="H448" s="3"/>
+    </row>
+    <row r="451" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+      <c r="A451" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F451" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="453" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A453" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F453" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="454" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="455" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A455" s="4"/>
+      <c r="B455" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C455" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F455" s="4"/>
+      <c r="G455" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H455" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="456" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A456" t="s">
+        <v>5</v>
+      </c>
+      <c r="B456">
+        <v>0.81838095238095199</v>
+      </c>
+      <c r="C456">
+        <v>0.7749659863945576</v>
+      </c>
+      <c r="F456" t="s">
+        <v>5</v>
+      </c>
+      <c r="G456">
+        <v>0.82247619047619003</v>
+      </c>
+      <c r="H456">
+        <v>0.77293877551020373</v>
+      </c>
+    </row>
+    <row r="457" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A457" t="s">
+        <v>9</v>
+      </c>
+      <c r="B457">
+        <v>2.7039823445212121E-3</v>
+      </c>
+      <c r="C457">
+        <v>2.8502530076069833E-3</v>
+      </c>
+      <c r="F457" t="s">
+        <v>9</v>
+      </c>
+      <c r="G457">
+        <v>2.4659372770924073E-3</v>
+      </c>
+      <c r="H457">
+        <v>3.1408309755992427E-3</v>
+      </c>
+    </row>
+    <row r="458" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A458" t="s">
+        <v>10</v>
+      </c>
+      <c r="B458">
+        <v>30</v>
+      </c>
+      <c r="C458">
+        <v>30</v>
+      </c>
+      <c r="F458" t="s">
+        <v>10</v>
+      </c>
+      <c r="G458">
+        <v>30</v>
+      </c>
+      <c r="H458">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="459" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A459" t="s">
+        <v>11</v>
+      </c>
+      <c r="B459">
+        <v>0.7912232360615068</v>
+      </c>
+      <c r="F459" t="s">
+        <v>11</v>
+      </c>
+      <c r="G459">
+        <v>0.81356298797537074</v>
+      </c>
+    </row>
+    <row r="460" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A460" t="s">
+        <v>12</v>
+      </c>
+      <c r="B460">
+        <v>0</v>
+      </c>
+      <c r="F460" t="s">
+        <v>12</v>
+      </c>
+      <c r="G460">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="461" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A461" t="s">
+        <v>13</v>
+      </c>
+      <c r="B461">
+        <v>29</v>
+      </c>
+      <c r="F461" t="s">
+        <v>13</v>
+      </c>
+      <c r="G461">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="462" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A462" t="s">
+        <v>14</v>
+      </c>
+      <c r="B462">
+        <v>6.9784929029714906</v>
+      </c>
+      <c r="F462" t="s">
+        <v>14</v>
+      </c>
+      <c r="G462">
+        <v>8.2620682637974276</v>
+      </c>
+    </row>
+    <row r="463" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A463" t="s">
+        <v>15</v>
+      </c>
+      <c r="B463">
+        <v>5.6641412676033006E-8</v>
+      </c>
+      <c r="F463" t="s">
+        <v>15</v>
+      </c>
+      <c r="G463">
+        <v>2.0734167435141375E-9</v>
+      </c>
+    </row>
+    <row r="464" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A464" t="s">
+        <v>16</v>
+      </c>
+      <c r="B464">
+        <v>1.6991270265334986</v>
+      </c>
+      <c r="F464" t="s">
+        <v>16</v>
+      </c>
+      <c r="G464">
+        <v>1.6991270265334986</v>
+      </c>
+    </row>
+    <row r="465" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A465" t="s">
+        <v>17</v>
+      </c>
+      <c r="B465">
+        <v>1.1328282535206601E-7</v>
+      </c>
+      <c r="F465" t="s">
+        <v>17</v>
+      </c>
+      <c r="G465">
+        <v>4.1468334870282749E-9</v>
+      </c>
+    </row>
+    <row r="466" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A466" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B466" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="C466" s="3"/>
+      <c r="F466" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G466" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="H466" s="3"/>
+    </row>
+    <row r="469" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+      <c r="A469" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F469" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="471" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A471" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F471" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="472" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="473" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A473" s="4"/>
+      <c r="B473" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C473" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F473" s="4"/>
+      <c r="G473" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H473" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="474" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A474" t="s">
+        <v>5</v>
+      </c>
+      <c r="B474">
+        <v>0.81838095238095199</v>
+      </c>
+      <c r="C474">
+        <v>0.82934693877550969</v>
+      </c>
+      <c r="F474" t="s">
+        <v>5</v>
+      </c>
+      <c r="G474">
+        <v>0.82247619047619003</v>
+      </c>
+      <c r="H474">
+        <v>0.82934693877550969</v>
+      </c>
+    </row>
+    <row r="475" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A475" t="s">
+        <v>9</v>
+      </c>
+      <c r="B475">
+        <v>2.7039823445212121E-3</v>
+      </c>
+      <c r="C475">
+        <v>2.2451949618693414E-3</v>
+      </c>
+      <c r="F475" t="s">
+        <v>9</v>
+      </c>
+      <c r="G475">
+        <v>2.4659372770924073E-3</v>
+      </c>
+      <c r="H475">
+        <v>2.2451949618693414E-3</v>
+      </c>
+    </row>
+    <row r="476" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A476" t="s">
+        <v>10</v>
+      </c>
+      <c r="B476">
+        <v>30</v>
+      </c>
+      <c r="C476">
+        <v>30</v>
+      </c>
+      <c r="F476" t="s">
+        <v>10</v>
+      </c>
+      <c r="G476">
+        <v>30</v>
+      </c>
+      <c r="H476">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="477" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A477" t="s">
+        <v>11</v>
+      </c>
+      <c r="B477">
+        <v>0.77425448405038644</v>
+      </c>
+      <c r="F477" t="s">
+        <v>11</v>
+      </c>
+      <c r="G477">
+        <v>0.80528104370980735</v>
+      </c>
+    </row>
+    <row r="478" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A478" t="s">
+        <v>12</v>
+      </c>
+      <c r="B478">
+        <v>0</v>
+      </c>
+      <c r="F478" t="s">
+        <v>12</v>
+      </c>
+      <c r="G478">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="479" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A479" t="s">
+        <v>13</v>
+      </c>
+      <c r="B479">
+        <v>29</v>
+      </c>
+      <c r="F479" t="s">
+        <v>13</v>
+      </c>
+      <c r="G479">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="480" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A480" t="s">
+        <v>14</v>
+      </c>
+      <c r="B480">
+        <v>-1.7838109808989098</v>
+      </c>
+      <c r="F480" t="s">
+        <v>14</v>
+      </c>
+      <c r="G480">
+        <v>-1.2396920173101287</v>
+      </c>
+    </row>
+    <row r="481" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A481" t="s">
+        <v>15</v>
+      </c>
+      <c r="B481">
+        <v>4.2461613043489478E-2</v>
+      </c>
+      <c r="F481" t="s">
+        <v>15</v>
+      </c>
+      <c r="G481">
+        <v>0.11251388531577002</v>
+      </c>
+    </row>
+    <row r="482" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A482" t="s">
+        <v>16</v>
+      </c>
+      <c r="B482">
+        <v>1.6991270265334986</v>
+      </c>
+      <c r="F482" t="s">
+        <v>16</v>
+      </c>
+      <c r="G482">
+        <v>1.6991270265334986</v>
+      </c>
+    </row>
+    <row r="483" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A483" t="s">
+        <v>17</v>
+      </c>
+      <c r="B483">
+        <v>8.4923226086978956E-2</v>
+      </c>
+      <c r="F483" t="s">
+        <v>17</v>
+      </c>
+      <c r="G483">
+        <v>0.22502777063154003</v>
+      </c>
+    </row>
+    <row r="484" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A484" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B484" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="C484" s="3"/>
+      <c r="F484" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G484" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="H484" s="3"/>
+    </row>
+    <row r="487" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+      <c r="A487" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F487" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="489" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A489" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F489" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="490" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="491" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A491" s="4"/>
+      <c r="B491" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C491" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F491" s="4"/>
+      <c r="G491" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H491" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="492" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A492" t="s">
+        <v>5</v>
+      </c>
+      <c r="B492">
+        <v>0.81838095238095199</v>
+      </c>
+      <c r="C492">
+        <v>0.90304761904761865</v>
+      </c>
+      <c r="F492" t="s">
+        <v>5</v>
+      </c>
+      <c r="G492">
+        <v>0.82247619047619003</v>
+      </c>
+      <c r="H492">
+        <v>0.90440816326530571</v>
+      </c>
+    </row>
+    <row r="493" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A493" t="s">
+        <v>9</v>
+      </c>
+      <c r="B493">
+        <v>2.7039823445212121E-3</v>
+      </c>
+      <c r="C493">
+        <v>1.5703426254386223E-3</v>
+      </c>
+      <c r="F493" t="s">
+        <v>9</v>
+      </c>
+      <c r="G493">
+        <v>2.4659372770924073E-3</v>
+      </c>
+      <c r="H493">
+        <v>1.5541041807292822E-3</v>
+      </c>
+    </row>
+    <row r="494" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A494" t="s">
+        <v>10</v>
+      </c>
+      <c r="B494">
+        <v>30</v>
+      </c>
+      <c r="C494">
+        <v>30</v>
+      </c>
+      <c r="F494" t="s">
+        <v>10</v>
+      </c>
+      <c r="G494">
+        <v>30</v>
+      </c>
+      <c r="H494">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="495" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A495" t="s">
+        <v>11</v>
+      </c>
+      <c r="B495">
+        <v>0.76662349294431864</v>
+      </c>
+      <c r="F495" t="s">
+        <v>11</v>
+      </c>
+      <c r="G495">
+        <v>0.74061233128474468</v>
+      </c>
+    </row>
+    <row r="496" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A496" t="s">
+        <v>12</v>
+      </c>
+      <c r="B496">
+        <v>0</v>
+      </c>
+      <c r="F496" t="s">
+        <v>12</v>
+      </c>
+      <c r="G496">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="497" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A497" t="s">
+        <v>13</v>
+      </c>
+      <c r="B497">
+        <v>29</v>
+      </c>
+      <c r="F497" t="s">
+        <v>13</v>
+      </c>
+      <c r="G497">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="498" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A498" t="s">
+        <v>14</v>
+      </c>
+      <c r="B498">
+        <v>-13.888638635984142</v>
+      </c>
+      <c r="F498" t="s">
+        <v>14</v>
+      </c>
+      <c r="G498">
+        <v>-13.407180869410377</v>
+      </c>
+    </row>
+    <row r="499" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A499" t="s">
+        <v>15</v>
+      </c>
+      <c r="B499">
+        <v>1.202127644881413E-14</v>
+      </c>
+      <c r="F499" t="s">
+        <v>15</v>
+      </c>
+      <c r="G499">
+        <v>2.9263368159621043E-14</v>
+      </c>
+    </row>
+    <row r="500" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A500" t="s">
+        <v>16</v>
+      </c>
+      <c r="B500">
+        <v>1.6991270265334986</v>
+      </c>
+      <c r="F500" t="s">
+        <v>16</v>
+      </c>
+      <c r="G500">
+        <v>1.6991270265334986</v>
+      </c>
+    </row>
+    <row r="501" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A501" t="s">
+        <v>17</v>
+      </c>
+      <c r="B501">
+        <v>2.404255289762826E-14</v>
+      </c>
+      <c r="F501" t="s">
+        <v>17</v>
+      </c>
+      <c r="G501">
+        <v>5.8526736319242086E-14</v>
+      </c>
+    </row>
+    <row r="502" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A502" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B502" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="C502" s="3"/>
+      <c r="F502" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G502" s="3">
+        <v>2.0452296421327048</v>
+      </c>
+      <c r="H502" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3944,15 +6969,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010090126F964B472F42BF44093AB6677E87" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e278873dc1fca5aa5836c9b4a4f7c188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="09d467f3-b700-42ea-8d14-5b9cd132b1f3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a263b2194a8338e0b3025a38ae8e56f9" ns3:_="">
     <xsd:import namespace="09d467f3-b700-42ea-8d14-5b9cd132b1f3"/>
@@ -4102,31 +7118,32 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B426A380-54CF-4D3F-B6FD-4C6030F40DB2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="09d467f3-b700-42ea-8d14-5b9cd132b1f3"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="09d467f3-b700-42ea-8d14-5b9cd132b1f3"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809DEFAF-712E-488F-A95B-AC80886515D9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C666C752-3E69-42FD-B366-A8C838657D31}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4144,6 +7161,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809DEFAF-712E-488F-A95B-AC80886515D9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{ec37a091-b9a6-47e5-98d0-903d4a419203}" enabled="0" method="" siteId="{ec37a091-b9a6-47e5-98d0-903d4a419203}" removed="1"/>

</xml_diff>

<commit_message>
Clean Up Format and Typos
</commit_message>
<xml_diff>
--- a/Results and Summary/CSCI 485 Final Project.xlsx
+++ b/Results and Summary/CSCI 485 Final Project.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Afolabi Soetan\Downloads\New folder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/83d3d0baac882484/Documents/CSCI 485 Final Project/Results and Summary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D33383B-BF29-4E58-B1C3-36F9FF737DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{2D33383B-BF29-4E58-B1C3-36F9FF737DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45EC227F-C199-4CAC-8257-9EE60DBDE745}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{AE118680-53F8-4A27-8AA4-2F3A3E8EE08C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17880" xr2:uid="{AE118680-53F8-4A27-8AA4-2F3A3E8EE08C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -333,10 +333,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4016,13 +4012,13 @@
       <c r="A272" t="s">
         <v>0</v>
       </c>
-      <c r="B272" t="s">
-        <v>22</v>
+      <c r="B272" s="2" t="s">
+        <v>1</v>
       </c>
       <c r="F272" t="s">
         <v>0</v>
       </c>
-      <c r="G272" t="s">
+      <c r="G272" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -4537,13 +4533,13 @@
         <v>5</v>
       </c>
       <c r="B303">
-        <v>0.78859999999999997</v>
+        <v>0.78649999999999998</v>
       </c>
       <c r="F303" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G303">
-        <v>0.78649999999999998</v>
+        <v>0.78859999999999997</v>
       </c>
     </row>
     <row r="306" spans="1:17" ht="21" x14ac:dyDescent="0.35">
@@ -4561,13 +4557,13 @@
       <c r="A308" t="s">
         <v>0</v>
       </c>
-      <c r="B308" t="s">
+      <c r="B308" s="2" t="s">
         <v>1</v>
       </c>
       <c r="F308" t="s">
         <v>0</v>
       </c>
-      <c r="G308" t="s">
+      <c r="G308" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -6969,6 +6965,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010090126F964B472F42BF44093AB6677E87" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e278873dc1fca5aa5836c9b4a4f7c188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="09d467f3-b700-42ea-8d14-5b9cd132b1f3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a263b2194a8338e0b3025a38ae8e56f9" ns3:_="">
     <xsd:import namespace="09d467f3-b700-42ea-8d14-5b9cd132b1f3"/>
@@ -7118,15 +7123,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B426A380-54CF-4D3F-B6FD-4C6030F40DB2}">
   <ds:schemaRefs>
@@ -7144,6 +7140,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809DEFAF-712E-488F-A95B-AC80886515D9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C666C752-3E69-42FD-B366-A8C838657D31}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7161,14 +7165,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809DEFAF-712E-488F-A95B-AC80886515D9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{ec37a091-b9a6-47e5-98d0-903d4a419203}" enabled="0" method="" siteId="{ec37a091-b9a6-47e5-98d0-903d4a419203}" removed="1"/>

</xml_diff>